<commit_message>
Finalize Part I and Part II notebooks and stabilize project pipeline
</commit_message>
<xml_diff>
--- a/outputs/Part_I_results_filled.xlsx
+++ b/outputs/Part_I_results_filled.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,25 +439,20 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Annualized Risk-Free Rate</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
           <t>Sharpe Ratio</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Minimum Monthly Return</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Maximum Monthly Return</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Total Cumulative Return</t>
         </is>
@@ -470,25 +465,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.07875194729931106</v>
+        <v>0.07875194570997557</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1080748036868332</v>
+        <v>0.1080748035952949</v>
       </c>
       <c r="D2" t="n">
-        <v>0.01754563106796116</v>
+        <v>0.5669864174765276</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5663328929905492</v>
+        <v>-0.07469915291397239</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.07469915412113819</v>
+        <v>0.1367273068063817</v>
       </c>
       <c r="G2" t="n">
-        <v>0.13672730681815</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1.395635548542889</v>
+        <v>1.395635503375626</v>
       </c>
     </row>
     <row r="3">
@@ -504,18 +496,15 @@
         <v>0.1567724004422423</v>
       </c>
       <c r="D3" t="n">
-        <v>0.01754563106796116</v>
+        <v>0.4087992013768466</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4083486688356475</v>
+        <v>-0.1676063446518038</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.1676063446518038</v>
+        <v>0.1344288672572242</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1344288672572242</v>
-      </c>
-      <c r="H3" t="n">
         <v>1.291800663892874</v>
       </c>
     </row>
@@ -555,7 +544,7 @@
         <v>41670</v>
       </c>
       <c r="B2" t="n">
-        <v>-0.03649865395696385</v>
+        <v>-0.03649865416421228</v>
       </c>
       <c r="C2" t="n">
         <v>-0.07026498004277006</v>
@@ -566,7 +555,7 @@
         <v>41698</v>
       </c>
       <c r="B3" t="n">
-        <v>0.01965962031856085</v>
+        <v>0.01965962026518523</v>
       </c>
       <c r="C3" t="n">
         <v>0.02077622686678488</v>
@@ -577,7 +566,7 @@
         <v>41729</v>
       </c>
       <c r="B4" t="n">
-        <v>0.01553912799890607</v>
+        <v>0.0155391281256913</v>
       </c>
       <c r="C4" t="n">
         <v>0.04467723574102896</v>
@@ -588,7 +577,7 @@
         <v>41759</v>
       </c>
       <c r="B5" t="n">
-        <v>0.02734641304080924</v>
+        <v>0.02734641306038766</v>
       </c>
       <c r="C5" t="n">
         <v>0.006795170125112241</v>
@@ -599,7 +588,7 @@
         <v>41789</v>
       </c>
       <c r="B6" t="n">
-        <v>0.006262336560474385</v>
+        <v>0.006262336674770144</v>
       </c>
       <c r="C6" t="n">
         <v>0.04339620179990861</v>
@@ -610,7 +599,7 @@
         <v>41820</v>
       </c>
       <c r="B7" t="n">
-        <v>0.01320043866512655</v>
+        <v>0.01320043855385788</v>
       </c>
       <c r="C7" t="n">
         <v>0.03569530268075231</v>
@@ -621,7 +610,7 @@
         <v>41851</v>
       </c>
       <c r="B8" t="n">
-        <v>0.00634089418775552</v>
+        <v>0.00634089399497464</v>
       </c>
       <c r="C8" t="n">
         <v>-0.007361026260429289</v>
@@ -632,7 +621,7 @@
         <v>41880</v>
       </c>
       <c r="B9" t="n">
-        <v>0.0387712121249143</v>
+        <v>0.03877121196595493</v>
       </c>
       <c r="C9" t="n">
         <v>0.02463494349528241</v>
@@ -643,7 +632,7 @@
         <v>41912</v>
       </c>
       <c r="B10" t="n">
-        <v>-0.03050354375449974</v>
+        <v>-0.03050354350157332</v>
       </c>
       <c r="C10" t="n">
         <v>-0.07531135274733532</v>
@@ -654,7 +643,7 @@
         <v>41943</v>
       </c>
       <c r="B11" t="n">
-        <v>0.02281906801371494</v>
+        <v>0.02281906843041514</v>
       </c>
       <c r="C11" t="n">
         <v>0.00775658866595595</v>
@@ -665,7 +654,7 @@
         <v>41971</v>
       </c>
       <c r="B12" t="n">
-        <v>-0.01887228532562114</v>
+        <v>-0.01887228565706454</v>
       </c>
       <c r="C12" t="n">
         <v>-0.02126323916811964</v>
@@ -676,7 +665,7 @@
         <v>42004</v>
       </c>
       <c r="B13" t="n">
-        <v>-0.03116883437874123</v>
+        <v>-0.03116883433505653</v>
       </c>
       <c r="C13" t="n">
         <v>-0.06901007205913473</v>
@@ -687,7 +676,7 @@
         <v>42034</v>
       </c>
       <c r="B14" t="n">
-        <v>0.0137115262182554</v>
+        <v>0.01371152603973757</v>
       </c>
       <c r="C14" t="n">
         <v>0.007339331453900047</v>
@@ -698,7 +687,7 @@
         <v>42062</v>
       </c>
       <c r="B15" t="n">
-        <v>0.03508508431879268</v>
+        <v>0.03508508435636881</v>
       </c>
       <c r="C15" t="n">
         <v>0.04141390361404322</v>
@@ -709,7 +698,7 @@
         <v>42094</v>
       </c>
       <c r="B16" t="n">
-        <v>-0.0007744917301810142</v>
+        <v>-0.0007744917573539734</v>
       </c>
       <c r="C16" t="n">
         <v>-0.03181535717049088</v>
@@ -720,7 +709,7 @@
         <v>42124</v>
       </c>
       <c r="B17" t="n">
-        <v>0.02706826663122262</v>
+        <v>0.0270682666372253</v>
       </c>
       <c r="C17" t="n">
         <v>0.05520842262682887</v>
@@ -731,7 +720,7 @@
         <v>42153</v>
       </c>
       <c r="B18" t="n">
-        <v>-0.04631065917551878</v>
+        <v>-0.04631065920667646</v>
       </c>
       <c r="C18" t="n">
         <v>-0.04519396145635353</v>
@@ -742,7 +731,7 @@
         <v>42185</v>
       </c>
       <c r="B19" t="n">
-        <v>-0.02770413006778343</v>
+        <v>-0.0277041300910287</v>
       </c>
       <c r="C19" t="n">
         <v>-0.01671837114782021</v>
@@ -753,7 +742,7 @@
         <v>42216</v>
       </c>
       <c r="B20" t="n">
-        <v>0.01860379034188642</v>
+        <v>0.01860379034121998</v>
       </c>
       <c r="C20" t="n">
         <v>-0.05212452092794789</v>
@@ -764,7 +753,7 @@
         <v>42247</v>
       </c>
       <c r="B21" t="n">
-        <v>-0.07187086909009724</v>
+        <v>-0.07187086903754682</v>
       </c>
       <c r="C21" t="n">
         <v>-0.08464422338745563</v>
@@ -775,7 +764,7 @@
         <v>42277</v>
       </c>
       <c r="B22" t="n">
-        <v>-0.01833165775342299</v>
+        <v>-0.01833165785473283</v>
       </c>
       <c r="C22" t="n">
         <v>-0.02493133275277176</v>
@@ -786,7 +775,7 @@
         <v>42307</v>
       </c>
       <c r="B23" t="n">
-        <v>0.03511363678730488</v>
+        <v>0.03511363660085631</v>
       </c>
       <c r="C23" t="n">
         <v>0.06491029329859194</v>
@@ -797,7 +786,7 @@
         <v>42338</v>
       </c>
       <c r="B24" t="n">
-        <v>-0.02591029444436185</v>
+        <v>-0.02591029444208056</v>
       </c>
       <c r="C24" t="n">
         <v>-0.0357558144902735</v>
@@ -808,7 +797,7 @@
         <v>42369</v>
       </c>
       <c r="B25" t="n">
-        <v>-0.01596111877501052</v>
+        <v>-0.01596111878380158</v>
       </c>
       <c r="C25" t="n">
         <v>-0.02106535603086771</v>
@@ -819,7 +808,7 @@
         <v>42398</v>
       </c>
       <c r="B26" t="n">
-        <v>0.04473407084893805</v>
+        <v>0.04473406834969725</v>
       </c>
       <c r="C26" t="n">
         <v>-0.04230023559388479</v>
@@ -830,7 +819,7 @@
         <v>42429</v>
       </c>
       <c r="B27" t="n">
-        <v>-0.00243889489822054</v>
+        <v>-0.0024388990608279</v>
       </c>
       <c r="C27" t="n">
         <v>-0.0078763026838919</v>
@@ -841,7 +830,7 @@
         <v>42460</v>
       </c>
       <c r="B28" t="n">
-        <v>0.08147079559328299</v>
+        <v>0.08147079497264535</v>
       </c>
       <c r="C28" t="n">
         <v>0.1344288672572242</v>
@@ -852,7 +841,7 @@
         <v>42489</v>
       </c>
       <c r="B29" t="n">
-        <v>-0.0201409321380176</v>
+        <v>-0.02014093371819024</v>
       </c>
       <c r="C29" t="n">
         <v>0.019650899382275</v>
@@ -863,7 +852,7 @@
         <v>42521</v>
       </c>
       <c r="B30" t="n">
-        <v>0.009053826483847069</v>
+        <v>0.009053828166525842</v>
       </c>
       <c r="C30" t="n">
         <v>-0.03779392015602362</v>
@@ -874,7 +863,7 @@
         <v>42551</v>
       </c>
       <c r="B31" t="n">
-        <v>0.05887672949777369</v>
+        <v>0.05887672707655323</v>
       </c>
       <c r="C31" t="n">
         <v>0.04977529648158455</v>
@@ -885,7 +874,7 @@
         <v>42580</v>
       </c>
       <c r="B32" t="n">
-        <v>0.01973486261259125</v>
+        <v>0.01973485816907689</v>
       </c>
       <c r="C32" t="n">
         <v>0.04574271959133058</v>
@@ -896,7 +885,7 @@
         <v>42613</v>
       </c>
       <c r="B33" t="n">
-        <v>-0.01247481766669782</v>
+        <v>-0.01247481344690763</v>
       </c>
       <c r="C33" t="n">
         <v>0.02043609851042295</v>
@@ -907,7 +896,7 @@
         <v>42643</v>
       </c>
       <c r="B34" t="n">
-        <v>-0.005238919229533591</v>
+        <v>-0.005238919074118562</v>
       </c>
       <c r="C34" t="n">
         <v>0.007018885117639503</v>
@@ -918,7 +907,7 @@
         <v>42674</v>
       </c>
       <c r="B35" t="n">
-        <v>-0.04004794132650656</v>
+        <v>-0.0400479406719685</v>
       </c>
       <c r="C35" t="n">
         <v>0.008182529362591296</v>
@@ -929,7 +918,7 @@
         <v>42704</v>
       </c>
       <c r="B36" t="n">
-        <v>-0.07469915412113819</v>
+        <v>-0.07469915291397239</v>
       </c>
       <c r="C36" t="n">
         <v>-0.03732341822162155</v>
@@ -940,7 +929,7 @@
         <v>42734</v>
       </c>
       <c r="B37" t="n">
-        <v>-0.02434305354521402</v>
+        <v>-0.02434305449003699</v>
       </c>
       <c r="C37" t="n">
         <v>0.02032329511426291</v>
@@ -951,7 +940,7 @@
         <v>42766</v>
       </c>
       <c r="B38" t="n">
-        <v>0.01357608535985715</v>
+        <v>0.01357608550579243</v>
       </c>
       <c r="C38" t="n">
         <v>0.04727385709321499</v>
@@ -962,7 +951,7 @@
         <v>42794</v>
       </c>
       <c r="B39" t="n">
-        <v>0.04708600857154882</v>
+        <v>0.04708600796748979</v>
       </c>
       <c r="C39" t="n">
         <v>0.02665901511045048</v>
@@ -973,7 +962,7 @@
         <v>42825</v>
       </c>
       <c r="B40" t="n">
-        <v>0.0201892740589598</v>
+        <v>0.02018927446922038</v>
       </c>
       <c r="C40" t="n">
         <v>0.02028145574585162</v>
@@ -984,7 +973,7 @@
         <v>42853</v>
       </c>
       <c r="B41" t="n">
-        <v>0.0003715570334755685</v>
+        <v>0.0003715564497607129</v>
       </c>
       <c r="C41" t="n">
         <v>0.01158976941153002</v>
@@ -995,7 +984,7 @@
         <v>42886</v>
       </c>
       <c r="B42" t="n">
-        <v>0.05543237695496969</v>
+        <v>0.0554323768789813</v>
       </c>
       <c r="C42" t="n">
         <v>0.01504055287089303</v>
@@ -1006,7 +995,7 @@
         <v>42916</v>
       </c>
       <c r="B43" t="n">
-        <v>0.000901319387124734</v>
+        <v>0.0009013197658726451</v>
       </c>
       <c r="C43" t="n">
         <v>0.001160368965973042</v>
@@ -1017,7 +1006,7 @@
         <v>42947</v>
       </c>
       <c r="B44" t="n">
-        <v>0.01066299590610429</v>
+        <v>0.01066299611965773</v>
       </c>
       <c r="C44" t="n">
         <v>0.04799108027004863</v>
@@ -1028,7 +1017,7 @@
         <v>42978</v>
       </c>
       <c r="B45" t="n">
-        <v>-0.004607831285661605</v>
+        <v>-0.004607831124146113</v>
       </c>
       <c r="C45" t="n">
         <v>0.02768204362181925</v>
@@ -1039,7 +1028,7 @@
         <v>43007</v>
       </c>
       <c r="B46" t="n">
-        <v>0.007875082516075846</v>
+        <v>0.007875082940049287</v>
       </c>
       <c r="C46" t="n">
         <v>-0.00570725226602121</v>
@@ -1050,7 +1039,7 @@
         <v>43039</v>
       </c>
       <c r="B47" t="n">
-        <v>0.007307510293602354</v>
+        <v>0.007307510240592709</v>
       </c>
       <c r="C47" t="n">
         <v>0.03870562748930086</v>
@@ -1061,7 +1050,7 @@
         <v>43069</v>
       </c>
       <c r="B48" t="n">
-        <v>0.01364089392327828</v>
+        <v>0.01364089450924604</v>
       </c>
       <c r="C48" t="n">
         <v>-0.005876212524494721</v>
@@ -1072,7 +1061,7 @@
         <v>43098</v>
       </c>
       <c r="B49" t="n">
-        <v>0.0462815568710923</v>
+        <v>0.04628155692471259</v>
       </c>
       <c r="C49" t="n">
         <v>0.05104246015880655</v>
@@ -1083,7 +1072,7 @@
         <v>43131</v>
       </c>
       <c r="B50" t="n">
-        <v>0.03724321209674699</v>
+        <v>0.0372432126422939</v>
       </c>
       <c r="C50" t="n">
         <v>0.0893234684450967</v>
@@ -1094,7 +1083,7 @@
         <v>43159</v>
       </c>
       <c r="B51" t="n">
-        <v>-0.02618760614260785</v>
+        <v>-0.02618760419048109</v>
       </c>
       <c r="C51" t="n">
         <v>-0.04479130657071866</v>
@@ -1105,7 +1094,7 @@
         <v>43189</v>
       </c>
       <c r="B52" t="n">
-        <v>0.01900678232749568</v>
+        <v>0.01900678106808058</v>
       </c>
       <c r="C52" t="n">
         <v>-0.01880510215300218</v>
@@ -1116,7 +1105,7 @@
         <v>43220</v>
       </c>
       <c r="B53" t="n">
-        <v>-0.00282253112223207</v>
+        <v>-0.002822531344317912</v>
       </c>
       <c r="C53" t="n">
         <v>-0.0006726306147162645</v>
@@ -1127,7 +1116,7 @@
         <v>43251</v>
       </c>
       <c r="B54" t="n">
-        <v>-0.05550433384790956</v>
+        <v>-0.05550433232821735</v>
       </c>
       <c r="C54" t="n">
         <v>-0.04379614011242528</v>
@@ -1138,7 +1127,7 @@
         <v>43280</v>
       </c>
       <c r="B55" t="n">
-        <v>-0.034419906806723</v>
+        <v>-0.03441991477683013</v>
       </c>
       <c r="C55" t="n">
         <v>-0.03727713089984806</v>
@@ -1149,7 +1138,7 @@
         <v>43312</v>
       </c>
       <c r="B56" t="n">
-        <v>0.01491953128754385</v>
+        <v>0.01491953329812574</v>
       </c>
       <c r="C56" t="n">
         <v>0.03580369355824013</v>
@@ -1160,7 +1149,7 @@
         <v>43343</v>
       </c>
       <c r="B57" t="n">
-        <v>-0.009778613903010396</v>
+        <v>-0.009778611968786882</v>
       </c>
       <c r="C57" t="n">
         <v>-0.01683805800516765</v>
@@ -1171,7 +1160,7 @@
         <v>43371</v>
       </c>
       <c r="B58" t="n">
-        <v>0.009075954559004387</v>
+        <v>0.009075954163016309</v>
       </c>
       <c r="C58" t="n">
         <v>0.01082714347627491</v>
@@ -1182,7 +1171,7 @@
         <v>43404</v>
       </c>
       <c r="B59" t="n">
-        <v>-0.05253338333573024</v>
+        <v>-0.05253338545020794</v>
       </c>
       <c r="C59" t="n">
         <v>-0.08162448270734325</v>
@@ -1193,7 +1182,7 @@
         <v>43434</v>
       </c>
       <c r="B60" t="n">
-        <v>0.02153674033240482</v>
+        <v>0.02153674073488552</v>
       </c>
       <c r="C60" t="n">
         <v>0.03803461615174045</v>
@@ -1204,7 +1193,7 @@
         <v>43465</v>
       </c>
       <c r="B61" t="n">
-        <v>0.01953265045944296</v>
+        <v>0.01953264768293812</v>
       </c>
       <c r="C61" t="n">
         <v>-0.01726815205799227</v>
@@ -1215,7 +1204,7 @@
         <v>43496</v>
       </c>
       <c r="B62" t="n">
-        <v>0.03661054394851312</v>
+        <v>0.03661054386609895</v>
       </c>
       <c r="C62" t="n">
         <v>0.07603690863090601</v>
@@ -1226,7 +1215,7 @@
         <v>43524</v>
       </c>
       <c r="B63" t="n">
-        <v>0.0224028642232468</v>
+        <v>0.02240286231202886</v>
       </c>
       <c r="C63" t="n">
         <v>-0.001483284179754729</v>
@@ -1237,7 +1226,7 @@
         <v>43553</v>
       </c>
       <c r="B64" t="n">
-        <v>0.008917643194512815</v>
+        <v>0.008917643301495151</v>
       </c>
       <c r="C64" t="n">
         <v>0.01296987343877379</v>
@@ -1248,7 +1237,7 @@
         <v>43585</v>
       </c>
       <c r="B65" t="n">
-        <v>0.008073205005376517</v>
+        <v>0.008073205459912745</v>
       </c>
       <c r="C65" t="n">
         <v>0.02224224988959288</v>
@@ -1259,7 +1248,7 @@
         <v>43616</v>
       </c>
       <c r="B66" t="n">
-        <v>-0.01124132433488315</v>
+        <v>-0.01124132435997483</v>
       </c>
       <c r="C66" t="n">
         <v>-0.04731589556520111</v>
@@ -1270,7 +1259,7 @@
         <v>43644</v>
       </c>
       <c r="B67" t="n">
-        <v>0.0437354964628522</v>
+        <v>0.0437354968493094</v>
       </c>
       <c r="C67" t="n">
         <v>0.05641209010605747</v>
@@ -1281,7 +1270,7 @@
         <v>43677</v>
       </c>
       <c r="B68" t="n">
-        <v>-0.005286451188886107</v>
+        <v>-0.005286450978308898</v>
       </c>
       <c r="C68" t="n">
         <v>-0.01440008118544814</v>
@@ -1292,7 +1281,7 @@
         <v>43707</v>
       </c>
       <c r="B69" t="n">
-        <v>0.01914790200737383</v>
+        <v>0.01914790261286416</v>
       </c>
       <c r="C69" t="n">
         <v>-0.05710121097500874</v>
@@ -1303,7 +1292,7 @@
         <v>43738</v>
       </c>
       <c r="B70" t="n">
-        <v>0.02627845134126465</v>
+        <v>0.02627845191585233</v>
       </c>
       <c r="C70" t="n">
         <v>0.03038971883415154</v>
@@ -1314,7 +1303,7 @@
         <v>43769</v>
       </c>
       <c r="B71" t="n">
-        <v>0.02962166397401734</v>
+        <v>0.02962166351179261</v>
       </c>
       <c r="C71" t="n">
         <v>0.03558394552960962</v>
@@ -1325,7 +1314,7 @@
         <v>43798</v>
       </c>
       <c r="B72" t="n">
-        <v>-0.03493622520940308</v>
+        <v>-0.03493622720370018</v>
       </c>
       <c r="C72" t="n">
         <v>-0.01065678404993961</v>
@@ -1336,7 +1325,7 @@
         <v>43830</v>
       </c>
       <c r="B73" t="n">
-        <v>0.02927859994366654</v>
+        <v>0.02927859986571662</v>
       </c>
       <c r="C73" t="n">
         <v>0.07206738650110425</v>
@@ -1347,7 +1336,7 @@
         <v>43861</v>
       </c>
       <c r="B74" t="n">
-        <v>-0.02502836508559387</v>
+        <v>-0.0250283646518741</v>
       </c>
       <c r="C74" t="n">
         <v>-0.0482064756652078</v>
@@ -1358,7 +1347,7 @@
         <v>43889</v>
       </c>
       <c r="B75" t="n">
-        <v>-0.04248689185744259</v>
+        <v>-0.04248689147271349</v>
       </c>
       <c r="C75" t="n">
         <v>-0.06670323746131065</v>
@@ -1369,7 +1358,7 @@
         <v>43921</v>
       </c>
       <c r="B76" t="n">
-        <v>-0.05917456638001409</v>
+        <v>-0.05917456649142699</v>
       </c>
       <c r="C76" t="n">
         <v>-0.1676063446518038</v>
@@ -1380,7 +1369,7 @@
         <v>43951</v>
       </c>
       <c r="B77" t="n">
-        <v>0.1004174839562125</v>
+        <v>0.1004174840674992</v>
       </c>
       <c r="C77" t="n">
         <v>0.09985373784843675</v>
@@ -1391,7 +1380,7 @@
         <v>43980</v>
       </c>
       <c r="B78" t="n">
-        <v>0.0075609937143513</v>
+        <v>0.007560993390064456</v>
       </c>
       <c r="C78" t="n">
         <v>0.004247792471245068</v>
@@ -1402,7 +1391,7 @@
         <v>44012</v>
       </c>
       <c r="B79" t="n">
-        <v>0.06204307972071473</v>
+        <v>0.06204307974958587</v>
       </c>
       <c r="C79" t="n">
         <v>0.06678052775027224</v>
@@ -1413,7 +1402,7 @@
         <v>44043</v>
       </c>
       <c r="B80" t="n">
-        <v>0.0353919204283569</v>
+        <v>0.03539191987199439</v>
       </c>
       <c r="C80" t="n">
         <v>0.07069760291997175</v>
@@ -1424,7 +1413,7 @@
         <v>44074</v>
       </c>
       <c r="B81" t="n">
-        <v>-0.01487788983008512</v>
+        <v>-0.01487788946211403</v>
       </c>
       <c r="C81" t="n">
         <v>0.002963455062672685</v>
@@ -1435,7 +1424,7 @@
         <v>44104</v>
       </c>
       <c r="B82" t="n">
-        <v>-0.02709824906346938</v>
+        <v>-0.0270982497928306</v>
       </c>
       <c r="C82" t="n">
         <v>-0.01976019159151884</v>
@@ -1446,7 +1435,7 @@
         <v>44134</v>
       </c>
       <c r="B83" t="n">
-        <v>0.02527055541667522</v>
+        <v>0.02527055547972409</v>
       </c>
       <c r="C83" t="n">
         <v>0.02076694896278813</v>
@@ -1457,7 +1446,7 @@
         <v>44165</v>
       </c>
       <c r="B84" t="n">
-        <v>0.04997765734784302</v>
+        <v>0.04997765722030623</v>
       </c>
       <c r="C84" t="n">
         <v>0.1138726461826266</v>
@@ -1468,7 +1457,7 @@
         <v>44196</v>
       </c>
       <c r="B85" t="n">
-        <v>0.02952371269523235</v>
+        <v>0.02952371267760976</v>
       </c>
       <c r="C85" t="n">
         <v>0.0863300868375526</v>
@@ -1479,7 +1468,7 @@
         <v>44225</v>
       </c>
       <c r="B86" t="n">
-        <v>-0.01240642631692593</v>
+        <v>-0.01240642626033056</v>
       </c>
       <c r="C86" t="n">
         <v>0.0290323743679554</v>
@@ -1490,7 +1479,7 @@
         <v>44253</v>
       </c>
       <c r="B87" t="n">
-        <v>0.01294189871842352</v>
+        <v>0.01294189887641626</v>
       </c>
       <c r="C87" t="n">
         <v>0.0323510740028403</v>
@@ -1501,7 +1490,7 @@
         <v>44286</v>
       </c>
       <c r="B88" t="n">
-        <v>0.03742807533337852</v>
+        <v>0.03742807550493847</v>
       </c>
       <c r="C88" t="n">
         <v>0.001187989845889644</v>
@@ -1512,7 +1501,7 @@
         <v>44316</v>
       </c>
       <c r="B89" t="n">
-        <v>0.0005421060586704085</v>
+        <v>0.0005421055571272707</v>
       </c>
       <c r="C89" t="n">
         <v>0.0235277295748508</v>
@@ -1523,7 +1512,7 @@
         <v>44347</v>
       </c>
       <c r="B90" t="n">
-        <v>0.007174088778612199</v>
+        <v>0.007174088572342188</v>
       </c>
       <c r="C90" t="n">
         <v>0.03436338529690337</v>
@@ -1534,7 +1523,7 @@
         <v>44377</v>
       </c>
       <c r="B91" t="n">
-        <v>0.006665568933330828</v>
+        <v>0.006665569391887116</v>
       </c>
       <c r="C91" t="n">
         <v>-0.005238501108997855</v>
@@ -1545,7 +1534,7 @@
         <v>44407</v>
       </c>
       <c r="B92" t="n">
-        <v>-0.001684561263260503</v>
+        <v>-0.001684561433368849</v>
       </c>
       <c r="C92" t="n">
         <v>-0.04397554540412282</v>
@@ -1556,7 +1545,7 @@
         <v>44439</v>
       </c>
       <c r="B93" t="n">
-        <v>0.02320069800647107</v>
+        <v>0.02320069799601338</v>
       </c>
       <c r="C93" t="n">
         <v>0.03903511321882387</v>
@@ -1567,7 +1556,7 @@
         <v>44469</v>
       </c>
       <c r="B94" t="n">
-        <v>-0.008133471897806001</v>
+        <v>-0.00813347172338306</v>
       </c>
       <c r="C94" t="n">
         <v>-0.02352828398363307</v>
@@ -1578,7 +1567,7 @@
         <v>44498</v>
       </c>
       <c r="B95" t="n">
-        <v>0.01753800014135151</v>
+        <v>0.01753800021027732</v>
       </c>
       <c r="C95" t="n">
         <v>0.008119557267448457</v>
@@ -1589,7 +1578,7 @@
         <v>44530</v>
       </c>
       <c r="B96" t="n">
-        <v>-0.006138495555229107</v>
+        <v>-0.006138495822780811</v>
       </c>
       <c r="C96" t="n">
         <v>-0.03487057144530385</v>
@@ -1600,7 +1589,7 @@
         <v>44561</v>
       </c>
       <c r="B97" t="n">
-        <v>0.01908879113483927</v>
+        <v>0.01908879116143317</v>
       </c>
       <c r="C97" t="n">
         <v>0.03877293711315413</v>
@@ -1611,7 +1600,7 @@
         <v>44592</v>
       </c>
       <c r="B98" t="n">
-        <v>-0.004416279005414903</v>
+        <v>-0.0044162790328264</v>
       </c>
       <c r="C98" t="n">
         <v>0.002924092229436752</v>
@@ -1622,7 +1611,7 @@
         <v>44620</v>
       </c>
       <c r="B99" t="n">
-        <v>0.005929697768733611</v>
+        <v>0.005929697681808897</v>
       </c>
       <c r="C99" t="n">
         <v>-0.04678409171731265</v>
@@ -1633,7 +1622,7 @@
         <v>44651</v>
       </c>
       <c r="B100" t="n">
-        <v>0.002369401685986447</v>
+        <v>0.002369401647356605</v>
       </c>
       <c r="C100" t="n">
         <v>0.02160171429843119</v>
@@ -1644,7 +1633,7 @@
         <v>44680</v>
       </c>
       <c r="B101" t="n">
-        <v>-0.009432437930342357</v>
+        <v>-0.009432437794156326</v>
       </c>
       <c r="C101" t="n">
         <v>-0.04929689726997008</v>
@@ -1655,7 +1644,7 @@
         <v>44712</v>
       </c>
       <c r="B102" t="n">
-        <v>-0.003265109939313502</v>
+        <v>-0.00326510997410868</v>
       </c>
       <c r="C102" t="n">
         <v>0.009638364803493562</v>
@@ -1666,7 +1655,7 @@
         <v>44742</v>
       </c>
       <c r="B103" t="n">
-        <v>-0.03376211190046922</v>
+        <v>-0.03376211178309475</v>
       </c>
       <c r="C103" t="n">
         <v>-0.07940058726618622</v>
@@ -1677,7 +1666,7 @@
         <v>44771</v>
       </c>
       <c r="B104" t="n">
-        <v>0.007045676429648514</v>
+        <v>0.007045676376755605</v>
       </c>
       <c r="C104" t="n">
         <v>0.00225283218921265</v>
@@ -1688,7 +1677,7 @@
         <v>44804</v>
       </c>
       <c r="B105" t="n">
-        <v>-0.004344407335357057</v>
+        <v>-0.004344407317424614</v>
       </c>
       <c r="C105" t="n">
         <v>0.0194592200082402</v>
@@ -1699,7 +1688,7 @@
         <v>44834</v>
       </c>
       <c r="B106" t="n">
-        <v>-0.04716076526397222</v>
+        <v>-0.04716076525371982</v>
       </c>
       <c r="C106" t="n">
         <v>-0.1019411321476542</v>
@@ -1710,7 +1699,7 @@
         <v>44865</v>
       </c>
       <c r="B107" t="n">
-        <v>-0.02898275132140758</v>
+        <v>-0.02898275129818562</v>
       </c>
       <c r="C107" t="n">
         <v>0.001203819237218551</v>
@@ -1721,7 +1710,7 @@
         <v>44895</v>
       </c>
       <c r="B108" t="n">
-        <v>0.13672730681815</v>
+        <v>0.1367273068063817</v>
       </c>
       <c r="C108" t="n">
         <v>0.13016429684924</v>
@@ -1732,7 +1721,7 @@
         <v>44925</v>
       </c>
       <c r="B109" t="n">
-        <v>-0.03505579169136976</v>
+        <v>-0.03505579172725707</v>
       </c>
       <c r="C109" t="n">
         <v>-0.02161397376045171</v>
@@ -1743,7 +1732,7 @@
         <v>44957</v>
       </c>
       <c r="B110" t="n">
-        <v>0.0296920626657074</v>
+        <v>0.02969206256979659</v>
       </c>
       <c r="C110" t="n">
         <v>0.06590833620845173</v>
@@ -1754,7 +1743,7 @@
         <v>44985</v>
       </c>
       <c r="B111" t="n">
-        <v>-0.0003239716824527559</v>
+        <v>-0.0003239717758208166</v>
       </c>
       <c r="C111" t="n">
         <v>-0.04502747129102448</v>
@@ -1765,7 +1754,7 @@
         <v>45016</v>
       </c>
       <c r="B112" t="n">
-        <v>0.03433484291448198</v>
+        <v>0.03433484292635736</v>
       </c>
       <c r="C112" t="n">
         <v>0.03462702520974735</v>
@@ -1776,7 +1765,7 @@
         <v>45044</v>
       </c>
       <c r="B113" t="n">
-        <v>0.03284531927904573</v>
+        <v>0.0328453193394511</v>
       </c>
       <c r="C113" t="n">
         <v>0.006221408189294738</v>
@@ -1787,7 +1776,7 @@
         <v>45077</v>
       </c>
       <c r="B114" t="n">
-        <v>0.0211764259967715</v>
+        <v>0.02117642596643819</v>
       </c>
       <c r="C114" t="n">
         <v>-0.001498942229409791</v>
@@ -1798,7 +1787,7 @@
         <v>45107</v>
       </c>
       <c r="B115" t="n">
-        <v>0.002255221206841292</v>
+        <v>0.002255221227168348</v>
       </c>
       <c r="C115" t="n">
         <v>0.03338471222996842</v>
@@ -1809,7 +1798,7 @@
         <v>45138</v>
       </c>
       <c r="B116" t="n">
-        <v>0.02470330265404508</v>
+        <v>0.02470330263373569</v>
       </c>
       <c r="C116" t="n">
         <v>0.0403096139031283</v>
@@ -1820,7 +1809,7 @@
         <v>45169</v>
       </c>
       <c r="B117" t="n">
-        <v>-0.03108599775753644</v>
+        <v>-0.03108599772549688</v>
       </c>
       <c r="C117" t="n">
         <v>-0.04637740616986598</v>
@@ -1831,7 +1820,7 @@
         <v>45198</v>
       </c>
       <c r="B118" t="n">
-        <v>-0.01949458909061902</v>
+        <v>-0.0194945890245552</v>
       </c>
       <c r="C118" t="n">
         <v>-0.0131917396815385</v>
@@ -1842,7 +1831,7 @@
         <v>45230</v>
       </c>
       <c r="B119" t="n">
-        <v>-0.02266454828625836</v>
+        <v>-0.022664548253229</v>
       </c>
       <c r="C119" t="n">
         <v>-0.03193660996460233</v>
@@ -1853,7 +1842,7 @@
         <v>45260</v>
       </c>
       <c r="B120" t="n">
-        <v>0.06364275556750981</v>
+        <v>0.06364275547966883</v>
       </c>
       <c r="C120" t="n">
         <v>0.07971419850955186</v>
@@ -1864,7 +1853,7 @@
         <v>45289</v>
       </c>
       <c r="B121" t="n">
-        <v>0.03759026108932309</v>
+        <v>0.03759026104415096</v>
       </c>
       <c r="C121" t="n">
         <v>0.04703396367444367</v>
@@ -1875,7 +1864,7 @@
         <v>45322</v>
       </c>
       <c r="B122" t="n">
-        <v>-0.007217413914594</v>
+        <v>-0.007217413861557577</v>
       </c>
       <c r="C122" t="n">
         <v>-0.01585787527416958</v>
@@ -1886,7 +1875,7 @@
         <v>45351</v>
       </c>
       <c r="B123" t="n">
-        <v>-0.004342256364362072</v>
+        <v>-0.004342256575710102</v>
       </c>
       <c r="C123" t="n">
         <v>0.03022495642883836</v>
@@ -1897,7 +1886,7 @@
         <v>45380</v>
       </c>
       <c r="B124" t="n">
-        <v>-0.01953843358682639</v>
+        <v>-0.01953843393865837</v>
       </c>
       <c r="C124" t="n">
         <v>0.02917740961821971</v>
@@ -1908,7 +1897,7 @@
         <v>45412</v>
       </c>
       <c r="B125" t="n">
-        <v>0.01619223792464995</v>
+        <v>0.0161922377797206</v>
       </c>
       <c r="C125" t="n">
         <v>0.01123730081200413</v>
@@ -1919,7 +1908,7 @@
         <v>45443</v>
       </c>
       <c r="B126" t="n">
-        <v>0.008240642931672834</v>
+        <v>0.008240643323985029</v>
       </c>
       <c r="C126" t="n">
         <v>0.01648872644524583</v>
@@ -1930,7 +1919,7 @@
         <v>45471</v>
       </c>
       <c r="B127" t="n">
-        <v>-0.01724511209072544</v>
+        <v>-0.01724511257095454</v>
       </c>
       <c r="C127" t="n">
         <v>0.0007354646659207265</v>
@@ -1941,7 +1930,7 @@
         <v>45504</v>
       </c>
       <c r="B128" t="n">
-        <v>0.02113785141336661</v>
+        <v>0.02113785160145753</v>
       </c>
       <c r="C128" t="n">
         <v>0.003334579349555053</v>
@@ -1952,7 +1941,7 @@
         <v>45534</v>
       </c>
       <c r="B129" t="n">
-        <v>0.03598561707515507</v>
+        <v>0.035985617226017</v>
       </c>
       <c r="C129" t="n">
         <v>0.01638387548657119</v>
@@ -1963,7 +1952,7 @@
         <v>45565</v>
       </c>
       <c r="B130" t="n">
-        <v>0.05509212861079952</v>
+        <v>0.05509212824741899</v>
       </c>
       <c r="C130" t="n">
         <v>0.033666084053502</v>
@@ -1974,7 +1963,7 @@
         <v>45596</v>
       </c>
       <c r="B131" t="n">
-        <v>-0.008899447771733012</v>
+        <v>-0.008899448039595201</v>
       </c>
       <c r="C131" t="n">
         <v>-0.04458566957284057</v>
@@ -1985,7 +1974,7 @@
         <v>45625</v>
       </c>
       <c r="B132" t="n">
-        <v>-0.03019807265952832</v>
+        <v>-0.03019807292186837</v>
       </c>
       <c r="C132" t="n">
         <v>-0.02738335071421504</v>
@@ -1996,7 +1985,7 @@
         <v>45657</v>
       </c>
       <c r="B133" t="n">
-        <v>0.004458709267329563</v>
+        <v>0.004458709194749865</v>
       </c>
       <c r="C133" t="n">
         <v>-0.003693654035491267</v>
@@ -2007,7 +1996,7 @@
         <v>45688</v>
       </c>
       <c r="B134" t="n">
-        <v>-0.01012098238772375</v>
+        <v>-0.01012098237064429</v>
       </c>
       <c r="C134" t="n">
         <v>0.005809586069590342</v>
@@ -2018,7 +2007,7 @@
         <v>45716</v>
       </c>
       <c r="B135" t="n">
-        <v>0.001975471167465166</v>
+        <v>0.001975471124104984</v>
       </c>
       <c r="C135" t="n">
         <v>-0.01602392225709455</v>
@@ -2029,7 +2018,7 @@
         <v>45747</v>
       </c>
       <c r="B136" t="n">
-        <v>0.0119798227523798</v>
+        <v>0.01197982270640709</v>
       </c>
       <c r="C136" t="n">
         <v>0.02116303136744554</v>
@@ -2040,7 +2029,7 @@
         <v>45777</v>
       </c>
       <c r="B137" t="n">
-        <v>0.01107818093411083</v>
+        <v>0.01107818091885257</v>
       </c>
       <c r="C137" t="n">
         <v>0.01716310963292009</v>
@@ -2051,7 +2040,7 @@
         <v>45807</v>
       </c>
       <c r="B138" t="n">
-        <v>0.04087487678577695</v>
+        <v>0.0408748768225022</v>
       </c>
       <c r="C138" t="n">
         <v>0.04571108411379798</v>
@@ -2062,7 +2051,7 @@
         <v>45838</v>
       </c>
       <c r="B139" t="n">
-        <v>0.02695355156794078</v>
+        <v>0.02695355150691722</v>
       </c>
       <c r="C139" t="n">
         <v>0.05114499695263859</v>
@@ -2073,7 +2062,7 @@
         <v>45869</v>
       </c>
       <c r="B140" t="n">
-        <v>0.001105337523106104</v>
+        <v>0.001105337613598443</v>
       </c>
       <c r="C140" t="n">
         <v>0.01207650834328272</v>
@@ -2084,7 +2073,7 @@
         <v>45898</v>
       </c>
       <c r="B141" t="n">
-        <v>0.01548353081089248</v>
+        <v>0.01548353080167544</v>
       </c>
       <c r="C141" t="n">
         <v>0.009490382556151769</v>
@@ -2095,7 +2084,7 @@
         <v>45930</v>
       </c>
       <c r="B142" t="n">
-        <v>0.02771801353531576</v>
+        <v>0.02771801345839262</v>
       </c>
       <c r="C142" t="n">
         <v>0.05080959391353825</v>
@@ -2106,7 +2095,7 @@
         <v>45961</v>
       </c>
       <c r="B143" t="n">
-        <v>0.0307273311505363</v>
+        <v>0.03072733112833025</v>
       </c>
       <c r="C143" t="n">
         <v>0.0494642092634302</v>
@@ -2117,7 +2106,7 @@
         <v>45989</v>
       </c>
       <c r="B144" t="n">
-        <v>0.005776013101891433</v>
+        <v>0.005776013045626965</v>
       </c>
       <c r="C144" t="n">
         <v>-0.009290385971130546</v>
@@ -2128,7 +2117,7 @@
         <v>46022</v>
       </c>
       <c r="B145" t="n">
-        <v>0.01025740007933732</v>
+        <v>0.01025740003853813</v>
       </c>
       <c r="C145" t="n">
         <v>0.03121426216286869</v>

</xml_diff>